<commit_message>
Improve schedule validation and retrieval
</commit_message>
<xml_diff>
--- a/fake data/02_Lab_Equipment.xlsx
+++ b/fake data/02_Lab_Equipment.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re7dcf0e928bd4ad5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lab Directory" sheetId="2" r:id="R551f524bd9e44755"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Inventory" sheetId="3" r:id="R009e5d2d2ee14b83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maintenance Plan" sheetId="4" r:id="R7524b8e8fc664fbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="5" r:id="R022f8c5091234e23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R88d06f0241a840a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lab Directory" sheetId="2" r:id="Rcaadbe64ac1a435f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment Inventory" sheetId="3" r:id="R2a6ba15c026d4efc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maintenance Plan" sheetId="4" r:id="Ra58a92d657aa41ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="5" r:id="Rbdb4f61bd0664533"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -105,7 +105,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="21">
+  <x:cellXfs count="22">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -137,6 +137,9 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -147,7 +150,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -158,7 +161,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -168,7 +171,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -178,7 +181,7 @@
         <x:color rgb="FF17365D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDEBF7"/>
         </x:patternFill>
       </x:fill>
@@ -386,7 +389,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7616ba826c6b4f25"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0d901b6e2a6a4364"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -907,7 +910,7 @@
     <x:mergeCell ref="A25:K25"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dbf8a5d3bae4d79"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14ba87ce3eb445f6"/>
 </x:worksheet>
 </file>
 
@@ -1510,7 +1513,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4a63ae83df54567"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8954b3ccc83d4e97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4338,7 +4341,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R843bb3f5aa624db7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R622784e19c914750"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5815,7 +5818,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ca07a699add4594"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ee00f7f976547eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5896,12 +5899,12 @@
         <x:v>15 minutes after Periods 1, 2, and 3; 30 minutes after Period 4.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="20" customHeight="1">
-      <x:c r="A11" s="20" t="str">
+    <x:row r="11" ht="36" customHeight="1">
+      <x:c r="A11" s="21" t="str">
         <x:v>Shared courses</x:v>
       </x:c>
-      <x:c r="B11" s="20" t="str">
-        <x:v>Shared-course lectures may combine majors; tutorials/labs always remain major-specific.</x:v>
+      <x:c r="B11" s="21" t="str">
+        <x:v>Only lectures may combine majors. Tutorials and labs must be scheduled separately for one major and one cohort group.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
@@ -5919,7 +5922,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba0841e352da4510"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R877c2646f0c44a5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>